<commit_message>
Update QA documentation and project files
</commit_message>
<xml_diff>
--- a/04_Yetkili_Kullanıcı_Profile_Settings/4 - AU - PS.xlsx
+++ b/04_Yetkili_Kullanıcı_Profile_Settings/4 - AU - PS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bovay\Desktop\¨¨¨¨¨¨\PROJECTS\CV TASLAK\POWER PULSE - PROJE\PLANLAMA\04 - YETKİLİ KULLANICI - PROFİL AYARLARI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8137525C-4318-4B56-868A-93F2CE14D837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2869CDED-F9B7-45FA-BD1C-72F5A701652F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="12090" firstSheet="9" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4. GEREKSİNİM TAKİP MATRİSİ" sheetId="11" r:id="rId1"/>
@@ -1899,6 +1899,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -2087,18 +2099,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2490,21 +2490,21 @@
       <c r="A1" s="57" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="73" t="s">
+      <c r="B1" s="77" t="s">
         <v>241</v>
       </c>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
       <c r="H1" s="58"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="57" t="s">
         <v>137</v>
       </c>
-      <c r="B2" s="75" t="s">
+      <c r="B2" s="79" t="s">
         <v>155</v>
       </c>
-      <c r="C2" s="74"/>
+      <c r="C2" s="78"/>
       <c r="F2" s="59" t="s">
         <v>138</v>
       </c>
@@ -2517,11 +2517,11 @@
       <c r="A3" s="57" t="s">
         <v>139</v>
       </c>
-      <c r="B3" s="75" t="s">
+      <c r="B3" s="79" t="s">
         <v>153</v>
       </c>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
       <c r="F3" s="59" t="s">
         <v>140</v>
       </c>
@@ -2534,10 +2534,10 @@
       <c r="A4" s="57" t="s">
         <v>141</v>
       </c>
-      <c r="B4" s="76" t="s">
+      <c r="B4" s="80" t="s">
         <v>154</v>
       </c>
-      <c r="C4" s="76"/>
+      <c r="C4" s="80"/>
       <c r="F4" s="57" t="s">
         <v>142</v>
       </c>
@@ -2577,7 +2577,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="155" t="s">
+      <c r="A8" s="73" t="s">
         <v>157</v>
       </c>
       <c r="B8" s="64" t="s">
@@ -2603,7 +2603,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="58.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="155" t="s">
+      <c r="A9" s="73" t="s">
         <v>196</v>
       </c>
       <c r="B9" s="64" t="s">
@@ -2629,7 +2629,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" ht="60.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="155" t="s">
+      <c r="A10" s="73" t="s">
         <v>195</v>
       </c>
       <c r="B10" s="64" t="s">
@@ -2655,7 +2655,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="60.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="155" t="s">
+      <c r="A11" s="73" t="s">
         <v>194</v>
       </c>
       <c r="B11" s="64" t="s">
@@ -2681,7 +2681,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="64" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="155" t="s">
+      <c r="A12" s="73" t="s">
         <v>193</v>
       </c>
       <c r="B12" s="64" t="s">
@@ -2707,7 +2707,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="155" t="s">
+      <c r="A13" s="73" t="s">
         <v>192</v>
       </c>
       <c r="B13" s="64" t="s">
@@ -2733,7 +2733,7 @@
       </c>
     </row>
     <row r="14" spans="1:8" ht="65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="155" t="s">
+      <c r="A14" s="73" t="s">
         <v>191</v>
       </c>
       <c r="B14" s="64" t="s">
@@ -2759,7 +2759,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="64.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="155" t="s">
+      <c r="A15" s="73" t="s">
         <v>197</v>
       </c>
       <c r="B15" s="64" t="s">
@@ -2785,7 +2785,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="77" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="155" t="s">
+      <c r="A16" s="73" t="s">
         <v>190</v>
       </c>
       <c r="B16" s="64" t="s">
@@ -2811,7 +2811,7 @@
       </c>
     </row>
     <row r="17" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="155" t="s">
+      <c r="A17" s="73" t="s">
         <v>158</v>
       </c>
       <c r="B17" s="64" t="s">
@@ -2837,7 +2837,7 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="155" t="s">
+      <c r="A18" s="73" t="s">
         <v>159</v>
       </c>
       <c r="B18" s="64" t="s">
@@ -2863,7 +2863,7 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="65.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="155" t="s">
+      <c r="A19" s="73" t="s">
         <v>160</v>
       </c>
       <c r="B19" s="64" t="s">
@@ -2889,7 +2889,7 @@
       </c>
     </row>
     <row r="20" spans="1:8" ht="98" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="155" t="s">
+      <c r="A20" s="73" t="s">
         <v>161</v>
       </c>
       <c r="B20" s="64" t="s">
@@ -2915,7 +2915,7 @@
       </c>
     </row>
     <row r="21" spans="1:8" ht="88" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="155" t="s">
+      <c r="A21" s="73" t="s">
         <v>162</v>
       </c>
       <c r="B21" s="64" t="s">
@@ -2941,7 +2941,7 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="63" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="155" t="s">
+      <c r="A22" s="73" t="s">
         <v>163</v>
       </c>
       <c r="B22" s="64" t="s">
@@ -2967,7 +2967,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="155" t="s">
+      <c r="A23" s="73" t="s">
         <v>164</v>
       </c>
       <c r="B23" s="64" t="s">
@@ -2993,7 +2993,7 @@
       </c>
     </row>
     <row r="24" spans="1:8" ht="88.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="155" t="s">
+      <c r="A24" s="73" t="s">
         <v>189</v>
       </c>
       <c r="B24" s="64" t="s">
@@ -3019,7 +3019,7 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="88" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="155" t="s">
+      <c r="A25" s="73" t="s">
         <v>188</v>
       </c>
       <c r="B25" s="64" t="s">
@@ -3045,7 +3045,7 @@
       </c>
     </row>
     <row r="26" spans="1:8" ht="85.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="155" t="s">
+      <c r="A26" s="73" t="s">
         <v>187</v>
       </c>
       <c r="B26" s="64" t="s">
@@ -3071,7 +3071,7 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="155" t="s">
+      <c r="A27" s="73" t="s">
         <v>186</v>
       </c>
       <c r="B27" s="64" t="s">
@@ -3097,7 +3097,7 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="83.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="155" t="s">
+      <c r="A28" s="73" t="s">
         <v>185</v>
       </c>
       <c r="B28" s="64" t="s">
@@ -3123,7 +3123,7 @@
       </c>
     </row>
     <row r="29" spans="1:8" ht="90.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="155" t="s">
+      <c r="A29" s="73" t="s">
         <v>184</v>
       </c>
       <c r="B29" s="64" t="s">
@@ -3149,7 +3149,7 @@
       </c>
     </row>
     <row r="30" spans="1:8" ht="81.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="155" t="s">
+      <c r="A30" s="73" t="s">
         <v>183</v>
       </c>
       <c r="B30" s="64" t="s">
@@ -3175,7 +3175,7 @@
       </c>
     </row>
     <row r="31" spans="1:8" ht="99.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="155" t="s">
+      <c r="A31" s="73" t="s">
         <v>182</v>
       </c>
       <c r="B31" s="64" t="s">
@@ -3201,7 +3201,7 @@
       </c>
     </row>
     <row r="32" spans="1:8" ht="102" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="155" t="s">
+      <c r="A32" s="73" t="s">
         <v>247</v>
       </c>
       <c r="B32" s="64" t="s">
@@ -3227,7 +3227,7 @@
       </c>
     </row>
     <row r="33" spans="1:8" ht="93" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="155" t="s">
+      <c r="A33" s="73" t="s">
         <v>248</v>
       </c>
       <c r="B33" s="64" t="s">
@@ -3253,7 +3253,7 @@
       </c>
     </row>
     <row r="34" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="155" t="s">
+      <c r="A34" s="73" t="s">
         <v>249</v>
       </c>
       <c r="B34" s="64" t="s">
@@ -3279,7 +3279,7 @@
       </c>
     </row>
     <row r="35" spans="1:8" ht="82" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="155" t="s">
+      <c r="A35" s="73" t="s">
         <v>250</v>
       </c>
       <c r="B35" s="64" t="s">
@@ -3305,7 +3305,7 @@
       </c>
     </row>
     <row r="36" spans="1:8" ht="78.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="155" t="s">
+      <c r="A36" s="73" t="s">
         <v>251</v>
       </c>
       <c r="B36" s="64" t="s">
@@ -3331,7 +3331,7 @@
       </c>
     </row>
     <row r="37" spans="1:8" ht="88" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="155" t="s">
+      <c r="A37" s="73" t="s">
         <v>252</v>
       </c>
       <c r="B37" s="64" t="s">
@@ -3357,7 +3357,7 @@
       </c>
     </row>
     <row r="38" spans="1:8" ht="82" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="155" t="s">
+      <c r="A38" s="73" t="s">
         <v>253</v>
       </c>
       <c r="B38" s="64" t="s">
@@ -3383,7 +3383,7 @@
       </c>
     </row>
     <row r="39" spans="1:8" ht="106" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="155" t="s">
+      <c r="A39" s="73" t="s">
         <v>254</v>
       </c>
       <c r="B39" s="64" t="s">
@@ -3409,7 +3409,7 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="119.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="155" t="s">
+      <c r="A40" s="73" t="s">
         <v>255</v>
       </c>
       <c r="B40" s="64" t="s">
@@ -3435,7 +3435,7 @@
       </c>
     </row>
     <row r="41" spans="1:8" ht="84" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="155" t="s">
+      <c r="A41" s="73" t="s">
         <v>256</v>
       </c>
       <c r="B41" s="64" t="s">
@@ -3461,7 +3461,7 @@
       </c>
     </row>
     <row r="42" spans="1:8" ht="104.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="155" t="s">
+      <c r="A42" s="73" t="s">
         <v>257</v>
       </c>
       <c r="B42" s="64" t="s">
@@ -3487,7 +3487,7 @@
       </c>
     </row>
     <row r="43" spans="1:8" ht="106" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="155" t="s">
+      <c r="A43" s="73" t="s">
         <v>258</v>
       </c>
       <c r="B43" s="64" t="s">
@@ -3513,7 +3513,7 @@
       </c>
     </row>
     <row r="44" spans="1:8" ht="88.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="155" t="s">
+      <c r="A44" s="73" t="s">
         <v>259</v>
       </c>
       <c r="B44" s="64" t="s">
@@ -3539,7 +3539,7 @@
       </c>
     </row>
     <row r="45" spans="1:8" ht="114.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="155" t="s">
+      <c r="A45" s="73" t="s">
         <v>260</v>
       </c>
       <c r="B45" s="64" t="s">
@@ -3565,7 +3565,7 @@
       </c>
     </row>
     <row r="46" spans="1:8" ht="97.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="155" t="s">
+      <c r="A46" s="73" t="s">
         <v>261</v>
       </c>
       <c r="B46" s="64" t="s">
@@ -3591,7 +3591,7 @@
       </c>
     </row>
     <row r="47" spans="1:8" ht="79.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="155" t="s">
+      <c r="A47" s="73" t="s">
         <v>262</v>
       </c>
       <c r="B47" s="64" t="s">
@@ -3617,7 +3617,7 @@
       </c>
     </row>
     <row r="48" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="155" t="s">
+      <c r="A48" s="73" t="s">
         <v>206</v>
       </c>
       <c r="B48" s="64" t="s">
@@ -3643,7 +3643,7 @@
       </c>
     </row>
     <row r="49" spans="1:8" ht="68" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="155" t="s">
+      <c r="A49" s="73" t="s">
         <v>244</v>
       </c>
       <c r="B49" s="64" t="s">
@@ -3669,7 +3669,7 @@
       </c>
     </row>
     <row r="50" spans="1:8" ht="52" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="155" t="s">
+      <c r="A50" s="73" t="s">
         <v>207</v>
       </c>
       <c r="B50" s="64" t="s">
@@ -3695,7 +3695,7 @@
       </c>
     </row>
     <row r="51" spans="1:8" ht="77" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="155" t="s">
+      <c r="A51" s="73" t="s">
         <v>245</v>
       </c>
       <c r="B51" s="64" t="s">
@@ -3721,7 +3721,7 @@
       </c>
     </row>
     <row r="52" spans="1:8" ht="67" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="155" t="s">
+      <c r="A52" s="73" t="s">
         <v>208</v>
       </c>
       <c r="B52" s="64" t="s">
@@ -3747,7 +3747,7 @@
       </c>
     </row>
     <row r="53" spans="1:8" ht="67.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="155" t="s">
+      <c r="A53" s="73" t="s">
         <v>246</v>
       </c>
       <c r="B53" s="64" t="s">
@@ -3773,7 +3773,7 @@
       </c>
     </row>
     <row r="54" spans="1:8" ht="86" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="156" t="s">
+      <c r="A54" s="74" t="s">
         <v>263</v>
       </c>
       <c r="B54" s="64" t="s">
@@ -3799,7 +3799,7 @@
       </c>
     </row>
     <row r="55" spans="1:8" ht="75.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="155" t="s">
+      <c r="A55" s="73" t="s">
         <v>264</v>
       </c>
       <c r="B55" s="64" t="s">
@@ -3825,7 +3825,7 @@
       </c>
     </row>
     <row r="56" spans="1:8" ht="71" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="155" t="s">
+      <c r="A56" s="73" t="s">
         <v>265</v>
       </c>
       <c r="B56" s="64" t="s">
@@ -3851,7 +3851,7 @@
       </c>
     </row>
     <row r="57" spans="1:8" ht="76" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="155" t="s">
+      <c r="A57" s="73" t="s">
         <v>266</v>
       </c>
       <c r="B57" s="64" t="s">
@@ -3877,7 +3877,7 @@
       </c>
     </row>
     <row r="58" spans="1:8" ht="69" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="155" t="s">
+      <c r="A58" s="73" t="s">
         <v>267</v>
       </c>
       <c r="B58" s="64" t="s">
@@ -3903,7 +3903,7 @@
       </c>
     </row>
     <row r="59" spans="1:8" ht="77" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="155" t="s">
+      <c r="A59" s="73" t="s">
         <v>268</v>
       </c>
       <c r="B59" s="64" t="s">
@@ -3929,7 +3929,7 @@
       </c>
     </row>
     <row r="60" spans="1:8" ht="71.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="155" t="s">
+      <c r="A60" s="73" t="s">
         <v>269</v>
       </c>
       <c r="B60" s="64" t="s">
@@ -3955,7 +3955,7 @@
       </c>
     </row>
     <row r="61" spans="1:8" ht="77" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="155" t="s">
+      <c r="A61" s="73" t="s">
         <v>270</v>
       </c>
       <c r="B61" s="64" t="s">
@@ -3981,7 +3981,7 @@
       </c>
     </row>
     <row r="62" spans="1:8" ht="78" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="155" t="s">
+      <c r="A62" s="73" t="s">
         <v>271</v>
       </c>
       <c r="B62" s="64" t="s">
@@ -4007,7 +4007,7 @@
       </c>
     </row>
     <row r="63" spans="1:8" ht="111" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="155" t="s">
+      <c r="A63" s="73" t="s">
         <v>272</v>
       </c>
       <c r="B63" s="64" t="s">
@@ -4033,7 +4033,7 @@
       </c>
     </row>
     <row r="64" spans="1:8" ht="111.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="155" t="s">
+      <c r="A64" s="73" t="s">
         <v>273</v>
       </c>
       <c r="B64" s="64" t="s">
@@ -4059,7 +4059,7 @@
       </c>
     </row>
     <row r="65" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="155" t="s">
+      <c r="A65" s="73" t="s">
         <v>211</v>
       </c>
       <c r="B65" s="64" t="s">
@@ -4085,7 +4085,7 @@
       </c>
     </row>
     <row r="66" spans="1:8" ht="116.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="157" t="s">
+      <c r="A66" s="75" t="s">
         <v>212</v>
       </c>
       <c r="B66" s="64" t="s">
@@ -4111,7 +4111,7 @@
       </c>
     </row>
     <row r="67" spans="1:8" ht="117" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="155" t="s">
+      <c r="A67" s="73" t="s">
         <v>213</v>
       </c>
       <c r="B67" s="64" t="s">
@@ -4137,7 +4137,7 @@
       </c>
     </row>
     <row r="68" spans="1:8" ht="105.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="158" t="s">
+      <c r="A68" s="76" t="s">
         <v>214</v>
       </c>
       <c r="B68" s="64" t="s">
@@ -4163,7 +4163,7 @@
       </c>
     </row>
     <row r="69" spans="1:8" ht="107.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="155" t="s">
+      <c r="A69" s="73" t="s">
         <v>215</v>
       </c>
       <c r="B69" s="64" t="s">
@@ -4189,7 +4189,7 @@
       </c>
     </row>
     <row r="70" spans="1:8" ht="103" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="155" t="s">
+      <c r="A70" s="73" t="s">
         <v>216</v>
       </c>
       <c r="B70" s="64" t="s">
@@ -4215,7 +4215,7 @@
       </c>
     </row>
     <row r="71" spans="1:8" ht="91.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="155" t="s">
+      <c r="A71" s="73" t="s">
         <v>217</v>
       </c>
       <c r="B71" s="64" t="s">
@@ -4241,7 +4241,7 @@
       </c>
     </row>
     <row r="72" spans="1:8" ht="104.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="155" t="s">
+      <c r="A72" s="73" t="s">
         <v>218</v>
       </c>
       <c r="B72" s="56" t="s">
@@ -4267,7 +4267,7 @@
       </c>
     </row>
     <row r="73" spans="1:8" ht="102.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A73" s="155" t="s">
+      <c r="A73" s="73" t="s">
         <v>219</v>
       </c>
       <c r="B73" s="56" t="s">
@@ -4293,7 +4293,7 @@
       </c>
     </row>
     <row r="74" spans="1:8" ht="106" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A74" s="155" t="s">
+      <c r="A74" s="73" t="s">
         <v>220</v>
       </c>
       <c r="B74" s="56" t="s">
@@ -4319,7 +4319,7 @@
       </c>
     </row>
     <row r="75" spans="1:8" ht="110.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="155" t="s">
+      <c r="A75" s="73" t="s">
         <v>221</v>
       </c>
       <c r="B75" s="56" t="s">
@@ -4345,7 +4345,7 @@
       </c>
     </row>
     <row r="76" spans="1:8" ht="104.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="155" t="s">
+      <c r="A76" s="73" t="s">
         <v>222</v>
       </c>
       <c r="B76" s="56" t="s">
@@ -4371,7 +4371,7 @@
       </c>
     </row>
     <row r="77" spans="1:8" ht="102" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="155" t="s">
+      <c r="A77" s="73" t="s">
         <v>223</v>
       </c>
       <c r="B77" s="56" t="s">
@@ -4397,7 +4397,7 @@
       </c>
     </row>
     <row r="78" spans="1:8" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="155" t="s">
+      <c r="A78" s="73" t="s">
         <v>224</v>
       </c>
       <c r="B78" s="56" t="s">
@@ -4423,7 +4423,7 @@
       </c>
     </row>
     <row r="79" spans="1:8" ht="94.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="155" t="s">
+      <c r="A79" s="73" t="s">
         <v>225</v>
       </c>
       <c r="B79" s="56" t="s">
@@ -4449,7 +4449,7 @@
       </c>
     </row>
     <row r="80" spans="1:8" ht="98.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A80" s="155" t="s">
+      <c r="A80" s="73" t="s">
         <v>226</v>
       </c>
       <c r="B80" s="56" t="s">
@@ -4475,7 +4475,7 @@
       </c>
     </row>
     <row r="81" spans="1:8" ht="96.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A81" s="155" t="s">
+      <c r="A81" s="73" t="s">
         <v>227</v>
       </c>
       <c r="B81" s="56" t="s">
@@ -4501,7 +4501,7 @@
       </c>
     </row>
     <row r="82" spans="1:8" ht="117.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="155" t="s">
+      <c r="A82" s="73" t="s">
         <v>228</v>
       </c>
       <c r="B82" s="56" t="s">
@@ -4527,7 +4527,7 @@
       </c>
     </row>
     <row r="83" spans="1:8" ht="109" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A83" s="155" t="s">
+      <c r="A83" s="73" t="s">
         <v>229</v>
       </c>
       <c r="B83" s="56" t="s">
@@ -4587,25 +4587,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="84"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
+      <c r="E1" s="88"/>
+      <c r="F1" s="88"/>
+      <c r="G1" s="88"/>
+      <c r="H1" s="88"/>
+      <c r="I1" s="88"/>
+      <c r="J1" s="88"/>
       <c r="K1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="85" t="s">
+      <c r="L1" s="89" t="s">
         <v>135</v>
       </c>
-      <c r="M1" s="85"/>
+      <c r="M1" s="89"/>
     </row>
     <row r="2" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="35"/>
@@ -4622,10 +4622,10 @@
       <c r="L2" s="36"/>
     </row>
     <row r="3" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="85" t="s">
+      <c r="A3" s="89" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="85"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="36"/>
       <c r="D3" s="36"/>
       <c r="E3" s="53"/>
@@ -4637,10 +4637,10 @@
       <c r="K3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="L3" s="85" t="s">
+      <c r="L3" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="M3" s="85"/>
+      <c r="M3" s="89"/>
     </row>
     <row r="4" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="7"/>
@@ -4657,62 +4657,62 @@
       <c r="L4" s="7"/>
     </row>
     <row r="5" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="83" t="s">
+      <c r="A5" s="87" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="83"/>
-      <c r="C5" s="83"/>
-      <c r="D5" s="83"/>
-      <c r="E5" s="83"/>
-      <c r="F5" s="83"/>
-      <c r="G5" s="83"/>
-      <c r="H5" s="83"/>
-      <c r="I5" s="83"/>
-      <c r="J5" s="78" t="s">
+      <c r="B5" s="87"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="87"/>
+      <c r="G5" s="87"/>
+      <c r="H5" s="87"/>
+      <c r="I5" s="87"/>
+      <c r="J5" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="K5" s="78"/>
-      <c r="L5" s="78"/>
+      <c r="K5" s="82"/>
+      <c r="L5" s="82"/>
     </row>
     <row r="6" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="83" t="s">
+      <c r="A6" s="87" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="83"/>
-      <c r="C6" s="83"/>
-      <c r="D6" s="83"/>
-      <c r="E6" s="83"/>
-      <c r="F6" s="83"/>
-      <c r="G6" s="83"/>
-      <c r="H6" s="83"/>
-      <c r="I6" s="83"/>
-      <c r="J6" s="78" t="s">
+      <c r="B6" s="87"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="87"/>
+      <c r="E6" s="87"/>
+      <c r="F6" s="87"/>
+      <c r="G6" s="87"/>
+      <c r="H6" s="87"/>
+      <c r="I6" s="87"/>
+      <c r="J6" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="K6" s="78"/>
-      <c r="L6" s="78"/>
+      <c r="K6" s="82"/>
+      <c r="L6" s="82"/>
     </row>
     <row r="7" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="83" t="s">
+      <c r="A7" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="83"/>
-      <c r="D7" s="83"/>
-      <c r="E7" s="83"/>
-      <c r="F7" s="83"/>
-      <c r="G7" s="83"/>
-      <c r="H7" s="83"/>
-      <c r="I7" s="83"/>
-      <c r="J7" s="78" t="s">
+      <c r="B7" s="87"/>
+      <c r="C7" s="87"/>
+      <c r="D7" s="87"/>
+      <c r="E7" s="87"/>
+      <c r="F7" s="87"/>
+      <c r="G7" s="87"/>
+      <c r="H7" s="87"/>
+      <c r="I7" s="87"/>
+      <c r="J7" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="K7" s="78"/>
-      <c r="L7" s="78"/>
+      <c r="K7" s="82"/>
+      <c r="L7" s="82"/>
     </row>
     <row r="8" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="79"/>
-      <c r="B8" s="79"/>
+      <c r="A8" s="83"/>
+      <c r="B8" s="83"/>
       <c r="C8" s="39"/>
       <c r="D8" s="39"/>
       <c r="E8" s="54"/>
@@ -4720,9 +4720,9 @@
       <c r="G8" s="54"/>
       <c r="H8" s="54"/>
       <c r="I8" s="39"/>
-      <c r="J8" s="80"/>
-      <c r="K8" s="80"/>
-      <c r="L8" s="80"/>
+      <c r="J8" s="84"/>
+      <c r="K8" s="84"/>
+      <c r="L8" s="84"/>
     </row>
     <row r="9" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="40"/>
@@ -4739,26 +4739,26 @@
       <c r="L9" s="40"/>
     </row>
     <row r="10" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="81" t="s">
+      <c r="A10" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="81"/>
-      <c r="C10" s="81"/>
-      <c r="D10" s="81"/>
-      <c r="E10" s="81"/>
-      <c r="F10" s="81"/>
-      <c r="G10" s="81"/>
-      <c r="H10" s="81"/>
-      <c r="I10" s="81"/>
-      <c r="J10" s="81"/>
-      <c r="K10" s="81"/>
+      <c r="B10" s="85"/>
+      <c r="C10" s="85"/>
+      <c r="D10" s="85"/>
+      <c r="E10" s="85"/>
+      <c r="F10" s="85"/>
+      <c r="G10" s="85"/>
+      <c r="H10" s="85"/>
+      <c r="I10" s="85"/>
+      <c r="J10" s="85"/>
+      <c r="K10" s="85"/>
       <c r="L10" s="40"/>
     </row>
     <row r="11" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="143" t="s">
+      <c r="A11" s="147" t="s">
         <v>79</v>
       </c>
-      <c r="B11" s="144"/>
+      <c r="B11" s="148"/>
       <c r="C11" s="66" t="s">
         <v>75</v>
       </c>
@@ -4771,21 +4771,21 @@
       <c r="F11" s="66" t="s">
         <v>78</v>
       </c>
-      <c r="G11" s="142" t="s">
+      <c r="G11" s="146" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="142"/>
-      <c r="I11" s="142" t="s">
+      <c r="H11" s="146"/>
+      <c r="I11" s="146" t="s">
         <v>21</v>
       </c>
-      <c r="J11" s="142"/>
+      <c r="J11" s="146"/>
       <c r="K11" s="67" t="s">
         <v>83</v>
       </c>
       <c r="L11" s="40"/>
     </row>
     <row r="12" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="145" t="s">
+      <c r="A12" s="149" t="s">
         <v>92</v>
       </c>
       <c r="B12" s="41" t="s">
@@ -4797,17 +4797,17 @@
       </c>
       <c r="E12" s="41"/>
       <c r="F12" s="42"/>
-      <c r="G12" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="H12" s="140"/>
-      <c r="I12" s="141"/>
-      <c r="J12" s="141"/>
+      <c r="G12" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="H12" s="144"/>
+      <c r="I12" s="145"/>
+      <c r="J12" s="145"/>
       <c r="K12" s="68"/>
       <c r="L12" s="40"/>
     </row>
     <row r="13" spans="1:13" ht="17.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="147"/>
+      <c r="A13" s="151"/>
       <c r="B13" s="41" t="s">
         <v>81</v>
       </c>
@@ -4817,17 +4817,17 @@
       <c r="D13" s="41"/>
       <c r="E13" s="41"/>
       <c r="F13" s="42"/>
-      <c r="G13" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="H13" s="140"/>
-      <c r="I13" s="141"/>
-      <c r="J13" s="141"/>
+      <c r="G13" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="H13" s="144"/>
+      <c r="I13" s="145"/>
+      <c r="J13" s="145"/>
       <c r="K13" s="68"/>
       <c r="L13" s="40"/>
     </row>
     <row r="14" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="148" t="s">
+      <c r="A14" s="152" t="s">
         <v>93</v>
       </c>
       <c r="B14" s="41" t="s">
@@ -4839,17 +4839,17 @@
       </c>
       <c r="E14" s="41"/>
       <c r="F14" s="42"/>
-      <c r="G14" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="H14" s="140"/>
-      <c r="I14" s="141"/>
-      <c r="J14" s="141"/>
+      <c r="G14" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="H14" s="144"/>
+      <c r="I14" s="145"/>
+      <c r="J14" s="145"/>
       <c r="K14" s="68"/>
       <c r="L14" s="40"/>
     </row>
     <row r="15" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="150"/>
+      <c r="A15" s="154"/>
       <c r="B15" s="41" t="s">
         <v>81</v>
       </c>
@@ -4859,17 +4859,17 @@
       <c r="D15" s="43"/>
       <c r="E15" s="43"/>
       <c r="F15" s="42"/>
-      <c r="G15" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="H15" s="140"/>
-      <c r="I15" s="141"/>
-      <c r="J15" s="141"/>
+      <c r="G15" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="H15" s="144"/>
+      <c r="I15" s="145"/>
+      <c r="J15" s="145"/>
       <c r="K15" s="68"/>
       <c r="L15" s="40"/>
     </row>
     <row r="16" spans="1:13" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="145" t="s">
+      <c r="A16" s="149" t="s">
         <v>94</v>
       </c>
       <c r="B16" s="41" t="s">
@@ -4881,17 +4881,17 @@
       <c r="F16" s="52" t="s">
         <v>95</v>
       </c>
-      <c r="G16" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="H16" s="140"/>
-      <c r="I16" s="141"/>
-      <c r="J16" s="141"/>
+      <c r="G16" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="H16" s="144"/>
+      <c r="I16" s="145"/>
+      <c r="J16" s="145"/>
       <c r="K16" s="68"/>
       <c r="L16" s="40"/>
     </row>
     <row r="17" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="147"/>
+      <c r="A17" s="151"/>
       <c r="B17" s="41" t="s">
         <v>81</v>
       </c>
@@ -4901,258 +4901,258 @@
         <v>95</v>
       </c>
       <c r="F17" s="42"/>
-      <c r="G17" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="H17" s="140"/>
-      <c r="I17" s="141"/>
-      <c r="J17" s="141"/>
+      <c r="G17" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="H17" s="144"/>
+      <c r="I17" s="145"/>
+      <c r="J17" s="145"/>
       <c r="K17" s="68"/>
       <c r="L17" s="40"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A18" s="92" t="s">
+      <c r="A18" s="96" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="93"/>
-      <c r="C18" s="92" t="s">
+      <c r="B18" s="97"/>
+      <c r="C18" s="96" t="s">
         <v>91</v>
       </c>
-      <c r="D18" s="93"/>
-      <c r="E18" s="81" t="s">
+      <c r="D18" s="97"/>
+      <c r="E18" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="F18" s="81"/>
-      <c r="G18" s="81" t="s">
+      <c r="F18" s="85"/>
+      <c r="G18" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="H18" s="81"/>
-      <c r="I18" s="92" t="s">
+      <c r="H18" s="85"/>
+      <c r="I18" s="96" t="s">
         <v>83</v>
       </c>
-      <c r="J18" s="93"/>
+      <c r="J18" s="97"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A19" s="145" t="s">
+      <c r="A19" s="149" t="s">
         <v>88</v>
       </c>
       <c r="B19" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="C19" s="151" t="s">
+      <c r="C19" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="D19" s="152"/>
-      <c r="E19" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F19" s="140"/>
-      <c r="G19" s="81"/>
-      <c r="H19" s="81"/>
-      <c r="I19" s="89"/>
-      <c r="J19" s="90"/>
+      <c r="D19" s="156"/>
+      <c r="E19" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="144"/>
+      <c r="G19" s="85"/>
+      <c r="H19" s="85"/>
+      <c r="I19" s="93"/>
+      <c r="J19" s="94"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A20" s="146"/>
+      <c r="A20" s="150"/>
       <c r="B20" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="C20" s="151" t="s">
+      <c r="C20" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="D20" s="152"/>
-      <c r="E20" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F20" s="140"/>
-      <c r="G20" s="81"/>
-      <c r="H20" s="81"/>
-      <c r="I20" s="89"/>
-      <c r="J20" s="90"/>
+      <c r="D20" s="156"/>
+      <c r="E20" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F20" s="144"/>
+      <c r="G20" s="85"/>
+      <c r="H20" s="85"/>
+      <c r="I20" s="93"/>
+      <c r="J20" s="94"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A21" s="146"/>
+      <c r="A21" s="150"/>
       <c r="B21" s="41" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="151" t="s">
+      <c r="C21" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="D21" s="152"/>
-      <c r="E21" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F21" s="140"/>
-      <c r="G21" s="81"/>
-      <c r="H21" s="81"/>
-      <c r="I21" s="89"/>
-      <c r="J21" s="90"/>
+      <c r="D21" s="156"/>
+      <c r="E21" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F21" s="144"/>
+      <c r="G21" s="85"/>
+      <c r="H21" s="85"/>
+      <c r="I21" s="93"/>
+      <c r="J21" s="94"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A22" s="147"/>
+      <c r="A22" s="151"/>
       <c r="B22" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="C22" s="151" t="s">
+      <c r="C22" s="155" t="s">
         <v>126</v>
       </c>
-      <c r="D22" s="152"/>
-      <c r="E22" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F22" s="140"/>
-      <c r="G22" s="81"/>
-      <c r="H22" s="81"/>
-      <c r="I22" s="89"/>
-      <c r="J22" s="90"/>
+      <c r="D22" s="156"/>
+      <c r="E22" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22" s="144"/>
+      <c r="G22" s="85"/>
+      <c r="H22" s="85"/>
+      <c r="I22" s="93"/>
+      <c r="J22" s="94"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A23" s="148" t="s">
+      <c r="A23" s="152" t="s">
         <v>89</v>
       </c>
       <c r="B23" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="C23" s="151" t="s">
+      <c r="C23" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="D23" s="152"/>
-      <c r="E23" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F23" s="140"/>
-      <c r="G23" s="81"/>
-      <c r="H23" s="81"/>
-      <c r="I23" s="89"/>
-      <c r="J23" s="90"/>
+      <c r="D23" s="156"/>
+      <c r="E23" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F23" s="144"/>
+      <c r="G23" s="85"/>
+      <c r="H23" s="85"/>
+      <c r="I23" s="93"/>
+      <c r="J23" s="94"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A24" s="149"/>
+      <c r="A24" s="153"/>
       <c r="B24" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="C24" s="151" t="s">
+      <c r="C24" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="D24" s="152"/>
-      <c r="E24" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F24" s="140"/>
-      <c r="G24" s="81"/>
-      <c r="H24" s="81"/>
-      <c r="I24" s="89"/>
-      <c r="J24" s="90"/>
+      <c r="D24" s="156"/>
+      <c r="E24" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F24" s="144"/>
+      <c r="G24" s="85"/>
+      <c r="H24" s="85"/>
+      <c r="I24" s="93"/>
+      <c r="J24" s="94"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A25" s="149"/>
+      <c r="A25" s="153"/>
       <c r="B25" s="41" t="s">
         <v>85</v>
       </c>
-      <c r="C25" s="151" t="s">
+      <c r="C25" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="D25" s="152"/>
-      <c r="E25" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F25" s="140"/>
-      <c r="G25" s="81"/>
-      <c r="H25" s="81"/>
-      <c r="I25" s="89"/>
-      <c r="J25" s="90"/>
+      <c r="D25" s="156"/>
+      <c r="E25" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F25" s="144"/>
+      <c r="G25" s="85"/>
+      <c r="H25" s="85"/>
+      <c r="I25" s="93"/>
+      <c r="J25" s="94"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A26" s="150"/>
+      <c r="A26" s="154"/>
       <c r="B26" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="C26" s="151" t="s">
+      <c r="C26" s="155" t="s">
         <v>126</v>
       </c>
-      <c r="D26" s="152"/>
-      <c r="E26" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F26" s="140"/>
-      <c r="G26" s="81"/>
-      <c r="H26" s="81"/>
-      <c r="I26" s="153"/>
-      <c r="J26" s="154"/>
+      <c r="D26" s="156"/>
+      <c r="E26" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F26" s="144"/>
+      <c r="G26" s="85"/>
+      <c r="H26" s="85"/>
+      <c r="I26" s="157"/>
+      <c r="J26" s="158"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A27" s="145" t="s">
+      <c r="A27" s="149" t="s">
         <v>90</v>
       </c>
       <c r="B27" s="44" t="s">
         <v>87</v>
       </c>
-      <c r="C27" s="151" t="s">
+      <c r="C27" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="D27" s="152"/>
-      <c r="E27" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F27" s="140"/>
-      <c r="G27" s="81"/>
-      <c r="H27" s="81"/>
-      <c r="I27" s="89"/>
-      <c r="J27" s="90"/>
+      <c r="D27" s="156"/>
+      <c r="E27" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F27" s="144"/>
+      <c r="G27" s="85"/>
+      <c r="H27" s="85"/>
+      <c r="I27" s="93"/>
+      <c r="J27" s="94"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A28" s="146"/>
+      <c r="A28" s="150"/>
       <c r="B28" s="41" t="s">
         <v>84</v>
       </c>
-      <c r="C28" s="151" t="s">
+      <c r="C28" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="D28" s="152"/>
-      <c r="E28" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F28" s="140"/>
-      <c r="G28" s="81"/>
-      <c r="H28" s="81"/>
-      <c r="I28" s="89"/>
-      <c r="J28" s="90"/>
+      <c r="D28" s="156"/>
+      <c r="E28" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F28" s="144"/>
+      <c r="G28" s="85"/>
+      <c r="H28" s="85"/>
+      <c r="I28" s="93"/>
+      <c r="J28" s="94"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A29" s="146"/>
+      <c r="A29" s="150"/>
       <c r="B29" s="41" t="s">
         <v>85</v>
       </c>
-      <c r="C29" s="151" t="s">
+      <c r="C29" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="D29" s="152"/>
-      <c r="E29" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F29" s="140"/>
-      <c r="G29" s="81"/>
-      <c r="H29" s="81"/>
-      <c r="I29" s="89"/>
-      <c r="J29" s="90"/>
+      <c r="D29" s="156"/>
+      <c r="E29" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F29" s="144"/>
+      <c r="G29" s="85"/>
+      <c r="H29" s="85"/>
+      <c r="I29" s="93"/>
+      <c r="J29" s="94"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A30" s="147"/>
+      <c r="A30" s="151"/>
       <c r="B30" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="C30" s="151" t="s">
+      <c r="C30" s="155" t="s">
         <v>126</v>
       </c>
-      <c r="D30" s="152"/>
-      <c r="E30" s="140" t="s">
-        <v>95</v>
-      </c>
-      <c r="F30" s="140"/>
-      <c r="G30" s="81"/>
-      <c r="H30" s="81"/>
-      <c r="I30" s="89"/>
-      <c r="J30" s="90"/>
+      <c r="D30" s="156"/>
+      <c r="E30" s="144" t="s">
+        <v>95</v>
+      </c>
+      <c r="F30" s="144"/>
+      <c r="G30" s="85"/>
+      <c r="H30" s="85"/>
+      <c r="I30" s="93"/>
+      <c r="J30" s="94"/>
     </row>
   </sheetData>
   <mergeCells count="87">
@@ -5259,18 +5259,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="85" t="s">
+      <c r="E1" s="89" t="s">
         <v>128</v>
       </c>
-      <c r="F1" s="85"/>
+      <c r="F1" s="89"/>
     </row>
     <row r="2" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -5280,18 +5280,18 @@
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="85" t="s">
+      <c r="A3" s="89" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="85"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="5"/>
       <c r="D3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="85" t="s">
+      <c r="E3" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="85"/>
+      <c r="F3" s="89"/>
     </row>
     <row r="4" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="7"/>
@@ -5301,44 +5301,44 @@
       <c r="E4" s="7"/>
     </row>
     <row r="5" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="83" t="s">
+      <c r="A5" s="87" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="83"/>
-      <c r="C5" s="78" t="s">
+      <c r="B5" s="87"/>
+      <c r="C5" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="78"/>
-      <c r="E5" s="78"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="82"/>
     </row>
     <row r="6" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="83" t="s">
+      <c r="A6" s="87" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="83"/>
-      <c r="C6" s="78" t="s">
+      <c r="B6" s="87"/>
+      <c r="C6" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="78"/>
-      <c r="E6" s="78"/>
+      <c r="D6" s="82"/>
+      <c r="E6" s="82"/>
     </row>
     <row r="7" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="83" t="s">
+      <c r="A7" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="78" t="s">
+      <c r="B7" s="87"/>
+      <c r="C7" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="78"/>
-      <c r="E7" s="78"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
     </row>
     <row r="8" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="79"/>
-      <c r="B8" s="79"/>
-      <c r="C8" s="80"/>
-      <c r="D8" s="80"/>
-      <c r="E8" s="80"/>
+      <c r="A8" s="83"/>
+      <c r="B8" s="83"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="84"/>
+      <c r="E8" s="84"/>
     </row>
     <row r="9" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="8"/>
@@ -5348,19 +5348,19 @@
       <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="81" t="s">
+      <c r="A10" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="81"/>
-      <c r="C10" s="81"/>
+      <c r="B10" s="85"/>
+      <c r="C10" s="85"/>
       <c r="D10" s="14"/>
       <c r="E10" s="8"/>
     </row>
     <row r="11" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="82" t="s">
+      <c r="A11" s="86" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="82"/>
+      <c r="B11" s="86"/>
       <c r="C11" s="45" t="s">
         <v>95</v>
       </c>
@@ -5368,10 +5368,10 @@
       <c r="E11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="77" t="s">
+      <c r="A12" s="81" t="s">
         <v>198</v>
       </c>
-      <c r="B12" s="77"/>
+      <c r="B12" s="81"/>
       <c r="C12" s="45" t="s">
         <v>95</v>
       </c>
@@ -5379,10 +5379,10 @@
       <c r="E12" s="8"/>
     </row>
     <row r="13" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="77" t="s">
+      <c r="A13" s="81" t="s">
         <v>199</v>
       </c>
-      <c r="B13" s="77"/>
+      <c r="B13" s="81"/>
       <c r="C13" s="45" t="s">
         <v>95</v>
       </c>
@@ -5390,10 +5390,10 @@
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="88" t="s">
+      <c r="A14" s="92" t="s">
         <v>200</v>
       </c>
-      <c r="B14" s="87"/>
+      <c r="B14" s="91"/>
       <c r="C14" s="45" t="s">
         <v>95</v>
       </c>
@@ -5401,10 +5401,10 @@
       <c r="E14" s="8"/>
     </row>
     <row r="15" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="77" t="s">
+      <c r="A15" s="81" t="s">
         <v>201</v>
       </c>
-      <c r="B15" s="77"/>
+      <c r="B15" s="81"/>
       <c r="C15" s="45" t="s">
         <v>95</v>
       </c>
@@ -5412,10 +5412,10 @@
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="77" t="s">
+      <c r="A16" s="81" t="s">
         <v>202</v>
       </c>
-      <c r="B16" s="77"/>
+      <c r="B16" s="81"/>
       <c r="C16" s="45" t="s">
         <v>95</v>
       </c>
@@ -5423,10 +5423,10 @@
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="86" t="s">
+      <c r="A17" s="90" t="s">
         <v>203</v>
       </c>
-      <c r="B17" s="87"/>
+      <c r="B17" s="91"/>
       <c r="C17" s="45" t="s">
         <v>95</v>
       </c>
@@ -5434,10 +5434,10 @@
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="86" t="s">
+      <c r="A18" s="90" t="s">
         <v>204</v>
       </c>
-      <c r="B18" s="87"/>
+      <c r="B18" s="91"/>
       <c r="C18" s="45" t="s">
         <v>95</v>
       </c>
@@ -5445,10 +5445,10 @@
       <c r="E18" s="8"/>
     </row>
     <row r="19" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A19" s="86" t="s">
+      <c r="A19" s="90" t="s">
         <v>205</v>
       </c>
-      <c r="B19" s="87"/>
+      <c r="B19" s="91"/>
       <c r="C19" s="45" t="s">
         <v>95</v>
       </c>
@@ -5456,10 +5456,10 @@
       <c r="E19" s="8"/>
     </row>
     <row r="20" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A20" s="89" t="s">
+      <c r="A20" s="93" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="90"/>
+      <c r="B20" s="94"/>
       <c r="C20" s="45" t="s">
         <v>95</v>
       </c>
@@ -5467,10 +5467,10 @@
       <c r="E20" s="12"/>
     </row>
     <row r="21" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A21" s="86" t="s">
+      <c r="A21" s="90" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="87"/>
+      <c r="B21" s="91"/>
       <c r="C21" s="45" t="s">
         <v>95</v>
       </c>
@@ -5478,10 +5478,10 @@
       <c r="E21" s="12"/>
     </row>
     <row r="22" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="86" t="s">
+      <c r="A22" s="90" t="s">
         <v>29</v>
       </c>
-      <c r="B22" s="87"/>
+      <c r="B22" s="91"/>
       <c r="C22" s="45" t="s">
         <v>95</v>
       </c>
@@ -5489,10 +5489,10 @@
       <c r="E22" s="12"/>
     </row>
     <row r="23" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A23" s="86" t="s">
+      <c r="A23" s="90" t="s">
         <v>30</v>
       </c>
-      <c r="B23" s="87"/>
+      <c r="B23" s="91"/>
       <c r="C23" s="45" t="s">
         <v>95</v>
       </c>
@@ -5500,10 +5500,10 @@
       <c r="E23" s="12"/>
     </row>
     <row r="24" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A24" s="86" t="s">
+      <c r="A24" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="87"/>
+      <c r="B24" s="91"/>
       <c r="C24" s="45" t="s">
         <v>95</v>
       </c>
@@ -5511,10 +5511,10 @@
       <c r="E24" s="12"/>
     </row>
     <row r="25" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A25" s="86" t="s">
+      <c r="A25" s="90" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="87"/>
+      <c r="B25" s="91"/>
       <c r="C25" s="45" t="s">
         <v>95</v>
       </c>
@@ -5522,10 +5522,10 @@
       <c r="E25" s="12"/>
     </row>
     <row r="26" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A26" s="86" t="s">
+      <c r="A26" s="90" t="s">
         <v>33</v>
       </c>
-      <c r="B26" s="87"/>
+      <c r="B26" s="91"/>
       <c r="C26" s="45" t="s">
         <v>95</v>
       </c>
@@ -5533,15 +5533,15 @@
       <c r="E26" s="12"/>
     </row>
     <row r="27" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A27" s="86"/>
-      <c r="B27" s="87"/>
+      <c r="A27" s="90"/>
+      <c r="B27" s="91"/>
       <c r="C27" s="15"/>
       <c r="D27" s="12"/>
       <c r="E27" s="12"/>
     </row>
     <row r="28" spans="1:5" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A28" s="77"/>
-      <c r="B28" s="77"/>
+      <c r="A28" s="81"/>
+      <c r="B28" s="81"/>
       <c r="C28" s="15"/>
       <c r="D28" s="8"/>
       <c r="E28" s="8"/>
@@ -5597,19 +5597,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
+      <c r="D1" s="88"/>
       <c r="E1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="85" t="s">
+      <c r="F1" s="89" t="s">
         <v>129</v>
       </c>
-      <c r="G1" s="85"/>
+      <c r="G1" s="89"/>
     </row>
     <row r="2" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
@@ -5620,19 +5620,19 @@
       <c r="F2" s="4"/>
     </row>
     <row r="3" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="85" t="s">
+      <c r="A3" s="89" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="85"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="4"/>
       <c r="D3" s="10"/>
       <c r="E3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="85" t="s">
+      <c r="F3" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="85"/>
+      <c r="G3" s="89"/>
     </row>
     <row r="4" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="7"/>
@@ -5643,48 +5643,48 @@
       <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="83" t="s">
+      <c r="A5" s="87" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="83"/>
-      <c r="C5" s="78" t="s">
+      <c r="B5" s="87"/>
+      <c r="C5" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="78"/>
-      <c r="E5" s="78"/>
-      <c r="F5" s="78"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="82"/>
+      <c r="F5" s="82"/>
     </row>
     <row r="6" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="83" t="s">
+      <c r="A6" s="87" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="83"/>
-      <c r="C6" s="78" t="s">
+      <c r="B6" s="87"/>
+      <c r="C6" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="78"/>
-      <c r="E6" s="78"/>
-      <c r="F6" s="78"/>
+      <c r="D6" s="82"/>
+      <c r="E6" s="82"/>
+      <c r="F6" s="82"/>
     </row>
     <row r="7" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="83" t="s">
+      <c r="A7" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="78" t="s">
+      <c r="B7" s="87"/>
+      <c r="C7" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="78"/>
-      <c r="E7" s="78"/>
-      <c r="F7" s="78"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
+      <c r="F7" s="82"/>
     </row>
     <row r="8" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="79"/>
-      <c r="B8" s="79"/>
+      <c r="A8" s="83"/>
+      <c r="B8" s="83"/>
       <c r="C8" s="11"/>
-      <c r="D8" s="80"/>
-      <c r="E8" s="80"/>
-      <c r="F8" s="80"/>
+      <c r="D8" s="84"/>
+      <c r="E8" s="84"/>
+      <c r="F8" s="84"/>
     </row>
     <row r="9" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="12"/>
@@ -5695,10 +5695,10 @@
       <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="92" t="s">
+      <c r="A10" s="96" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="93"/>
+      <c r="B10" s="97"/>
       <c r="C10" s="13" t="s">
         <v>35</v>
       </c>
@@ -5711,10 +5711,10 @@
       <c r="F10" s="69"/>
     </row>
     <row r="11" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="82" t="s">
+      <c r="A11" s="86" t="s">
         <v>174</v>
       </c>
-      <c r="B11" s="82"/>
+      <c r="B11" s="86"/>
       <c r="C11" s="45" t="s">
         <v>95</v>
       </c>
@@ -5727,10 +5727,10 @@
       <c r="F11" s="70"/>
     </row>
     <row r="12" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="82" t="s">
+      <c r="A12" s="86" t="s">
         <v>175</v>
       </c>
-      <c r="B12" s="82"/>
+      <c r="B12" s="86"/>
       <c r="C12" s="45" t="s">
         <v>95</v>
       </c>
@@ -5743,10 +5743,10 @@
       <c r="F12" s="70"/>
     </row>
     <row r="13" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="91" t="s">
+      <c r="A13" s="95" t="s">
         <v>176</v>
       </c>
-      <c r="B13" s="90"/>
+      <c r="B13" s="94"/>
       <c r="C13" s="45" t="s">
         <v>95</v>
       </c>
@@ -5759,10 +5759,10 @@
       <c r="F13" s="70"/>
     </row>
     <row r="14" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="82" t="s">
+      <c r="A14" s="86" t="s">
         <v>177</v>
       </c>
-      <c r="B14" s="82"/>
+      <c r="B14" s="86"/>
       <c r="C14" s="45" t="s">
         <v>95</v>
       </c>
@@ -5775,10 +5775,10 @@
       <c r="F14" s="70"/>
     </row>
     <row r="15" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="82" t="s">
+      <c r="A15" s="86" t="s">
         <v>178</v>
       </c>
-      <c r="B15" s="82"/>
+      <c r="B15" s="86"/>
       <c r="C15" s="45" t="s">
         <v>95</v>
       </c>
@@ -5791,10 +5791,10 @@
       <c r="F15" s="70"/>
     </row>
     <row r="16" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="89" t="s">
+      <c r="A16" s="93" t="s">
         <v>179</v>
       </c>
-      <c r="B16" s="90"/>
+      <c r="B16" s="94"/>
       <c r="C16" s="45" t="s">
         <v>95</v>
       </c>
@@ -5807,10 +5807,10 @@
       <c r="F16" s="70"/>
     </row>
     <row r="17" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A17" s="89" t="s">
+      <c r="A17" s="93" t="s">
         <v>180</v>
       </c>
-      <c r="B17" s="90"/>
+      <c r="B17" s="94"/>
       <c r="C17" s="45" t="s">
         <v>95</v>
       </c>
@@ -5823,10 +5823,10 @@
       <c r="F17" s="70"/>
     </row>
     <row r="18" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A18" s="89" t="s">
+      <c r="A18" s="93" t="s">
         <v>181</v>
       </c>
-      <c r="B18" s="90"/>
+      <c r="B18" s="94"/>
       <c r="C18" s="45" t="s">
         <v>95</v>
       </c>
@@ -5888,94 +5888,94 @@
       <c r="C1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="97" t="s">
+      <c r="D1" s="101" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="99"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="103"/>
     </row>
     <row r="2" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="100" t="s">
+      <c r="B2" s="104" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="101"/>
+      <c r="C2" s="105"/>
       <c r="D2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="100" t="s">
+      <c r="E2" s="104" t="s">
         <v>97</v>
       </c>
-      <c r="F2" s="102"/>
-      <c r="G2" s="102"/>
-      <c r="H2" s="103"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="107"/>
     </row>
     <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="104" t="s">
+      <c r="A3" s="108" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="98"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="105"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98"/>
-      <c r="H3" s="99"/>
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="103"/>
     </row>
     <row r="4" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="19">
         <v>1</v>
       </c>
-      <c r="B4" s="94" t="s">
+      <c r="B4" s="98" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="96"/>
+      <c r="C4" s="99"/>
+      <c r="D4" s="99"/>
+      <c r="E4" s="99"/>
+      <c r="F4" s="99"/>
+      <c r="G4" s="99"/>
+      <c r="H4" s="100"/>
     </row>
     <row r="5" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="20">
         <v>2</v>
       </c>
-      <c r="B5" s="100" t="s">
+      <c r="B5" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="102"/>
-      <c r="D5" s="102"/>
-      <c r="E5" s="102"/>
-      <c r="F5" s="102"/>
-      <c r="G5" s="102"/>
-      <c r="H5" s="103"/>
+      <c r="C5" s="106"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="106"/>
+      <c r="F5" s="106"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="107"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="106" t="s">
+      <c r="A6" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="98"/>
-      <c r="C6" s="98"/>
-      <c r="D6" s="98"/>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98"/>
-      <c r="G6" s="98"/>
-      <c r="H6" s="99"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="102"/>
+      <c r="H6" s="103"/>
     </row>
     <row r="7" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="107" t="s">
+      <c r="A7" s="111" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="108"/>
-      <c r="C7" s="109"/>
-      <c r="D7" s="110" t="s">
+      <c r="B7" s="112"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="114" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="109"/>
+      <c r="E7" s="113"/>
       <c r="F7" s="50" t="s">
         <v>20</v>
       </c>
@@ -5990,14 +5990,14 @@
       <c r="A8" s="19">
         <v>1</v>
       </c>
-      <c r="B8" s="94" t="s">
+      <c r="B8" s="98" t="s">
         <v>71</v>
       </c>
-      <c r="C8" s="111"/>
-      <c r="D8" s="94" t="s">
+      <c r="C8" s="115"/>
+      <c r="D8" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E8" s="112"/>
+      <c r="E8" s="116"/>
       <c r="F8" s="46"/>
       <c r="G8" s="46" t="s">
         <v>96</v>
@@ -6010,14 +6010,14 @@
       <c r="A9" s="19">
         <v>2</v>
       </c>
-      <c r="B9" s="94" t="s">
+      <c r="B9" s="98" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="111"/>
-      <c r="D9" s="94" t="s">
+      <c r="C9" s="115"/>
+      <c r="D9" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E9" s="112"/>
+      <c r="E9" s="116"/>
       <c r="F9" s="21"/>
       <c r="G9" s="46" t="s">
         <v>96</v>
@@ -6030,14 +6030,14 @@
       <c r="A10" s="19">
         <v>3</v>
       </c>
-      <c r="B10" s="94" t="s">
+      <c r="B10" s="98" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="111"/>
-      <c r="D10" s="94" t="s">
+      <c r="C10" s="115"/>
+      <c r="D10" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E10" s="112"/>
+      <c r="E10" s="116"/>
       <c r="F10" s="46" t="s">
         <v>95</v>
       </c>
@@ -6048,14 +6048,14 @@
       <c r="A11" s="19">
         <v>4</v>
       </c>
-      <c r="B11" s="94" t="s">
+      <c r="B11" s="98" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="111"/>
-      <c r="D11" s="94" t="s">
+      <c r="C11" s="115"/>
+      <c r="D11" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E11" s="112"/>
+      <c r="E11" s="116"/>
       <c r="F11" s="46" t="s">
         <v>95</v>
       </c>
@@ -6066,14 +6066,14 @@
       <c r="A12" s="19">
         <v>5</v>
       </c>
-      <c r="B12" s="94" t="s">
+      <c r="B12" s="98" t="s">
         <v>46</v>
       </c>
-      <c r="C12" s="111"/>
-      <c r="D12" s="100" t="s">
+      <c r="C12" s="115"/>
+      <c r="D12" s="104" t="s">
         <v>243</v>
       </c>
-      <c r="E12" s="120"/>
+      <c r="E12" s="124"/>
       <c r="F12" s="46" t="s">
         <v>95</v>
       </c>
@@ -6084,14 +6084,14 @@
       <c r="A13" s="19">
         <v>6</v>
       </c>
-      <c r="B13" s="94" t="s">
+      <c r="B13" s="98" t="s">
         <v>240</v>
       </c>
-      <c r="C13" s="111"/>
-      <c r="D13" s="100" t="s">
+      <c r="C13" s="115"/>
+      <c r="D13" s="104" t="s">
         <v>243</v>
       </c>
-      <c r="E13" s="120"/>
+      <c r="E13" s="124"/>
       <c r="F13" s="46" t="s">
         <v>95</v>
       </c>
@@ -6102,14 +6102,14 @@
       <c r="A14" s="23">
         <v>7</v>
       </c>
-      <c r="B14" s="100" t="s">
+      <c r="B14" s="104" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="120"/>
-      <c r="D14" s="100" t="s">
+      <c r="C14" s="124"/>
+      <c r="D14" s="104" t="s">
         <v>243</v>
       </c>
-      <c r="E14" s="120"/>
+      <c r="E14" s="124"/>
       <c r="F14" s="46" t="s">
         <v>95</v>
       </c>
@@ -6117,22 +6117,22 @@
       <c r="H14" s="25"/>
     </row>
     <row r="15" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="113" t="s">
+      <c r="A15" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="114"/>
-      <c r="C15" s="115" t="s">
+      <c r="B15" s="118"/>
+      <c r="C15" s="119" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="116"/>
+      <c r="D15" s="120"/>
       <c r="E15" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F15" s="117">
+      <c r="F15" s="121">
         <v>46227</v>
       </c>
-      <c r="G15" s="118"/>
-      <c r="H15" s="119"/>
+      <c r="G15" s="122"/>
+      <c r="H15" s="123"/>
     </row>
   </sheetData>
   <mergeCells count="27">
@@ -6189,13 +6189,13 @@
       <c r="B1" s="47" t="s">
         <v>152</v>
       </c>
-      <c r="C1" s="126"/>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="127"/>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="127"/>
+      <c r="C1" s="130"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="131"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="47" t="s">
@@ -6211,11 +6211,11 @@
       <c r="E2" s="47" t="s">
         <v>101</v>
       </c>
-      <c r="F2" s="122" t="s">
+      <c r="F2" s="126" t="s">
         <v>125</v>
       </c>
-      <c r="G2" s="128"/>
-      <c r="H2" s="129"/>
+      <c r="G2" s="132"/>
+      <c r="H2" s="133"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="47" t="s">
@@ -6233,297 +6233,297 @@
       <c r="E3" s="47" t="s">
         <v>105</v>
       </c>
-      <c r="F3" s="122" t="s">
+      <c r="F3" s="126" t="s">
         <v>97</v>
       </c>
-      <c r="G3" s="128"/>
-      <c r="H3" s="129"/>
+      <c r="G3" s="132"/>
+      <c r="H3" s="133"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="47" t="s">
         <v>106</v>
       </c>
-      <c r="B4" s="122" t="s">
+      <c r="B4" s="126" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="128"/>
-      <c r="D4" s="128"/>
-      <c r="E4" s="128"/>
-      <c r="F4" s="128"/>
-      <c r="G4" s="128"/>
-      <c r="H4" s="129"/>
+      <c r="C4" s="132"/>
+      <c r="D4" s="132"/>
+      <c r="E4" s="132"/>
+      <c r="F4" s="132"/>
+      <c r="G4" s="132"/>
+      <c r="H4" s="133"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="47" t="s">
         <v>107</v>
       </c>
-      <c r="B5" s="121" t="s">
+      <c r="B5" s="125" t="s">
         <v>239</v>
       </c>
-      <c r="C5" s="121"/>
-      <c r="D5" s="121"/>
-      <c r="E5" s="121"/>
-      <c r="F5" s="121"/>
-      <c r="G5" s="121"/>
-      <c r="H5" s="121"/>
+      <c r="C5" s="125"/>
+      <c r="D5" s="125"/>
+      <c r="E5" s="125"/>
+      <c r="F5" s="125"/>
+      <c r="G5" s="125"/>
+      <c r="H5" s="125"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="47" t="s">
         <v>108</v>
       </c>
-      <c r="B6" s="121" t="s">
+      <c r="B6" s="125" t="s">
         <v>113</v>
       </c>
-      <c r="C6" s="121"/>
-      <c r="D6" s="121"/>
-      <c r="E6" s="121"/>
-      <c r="F6" s="121"/>
-      <c r="G6" s="121"/>
-      <c r="H6" s="121"/>
+      <c r="C6" s="125"/>
+      <c r="D6" s="125"/>
+      <c r="E6" s="125"/>
+      <c r="F6" s="125"/>
+      <c r="G6" s="125"/>
+      <c r="H6" s="125"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="122" t="s">
+      <c r="A7" s="126" t="s">
         <v>114</v>
       </c>
-      <c r="B7" s="123"/>
-      <c r="C7" s="123"/>
-      <c r="D7" s="123"/>
-      <c r="E7" s="123"/>
-      <c r="F7" s="123"/>
-      <c r="G7" s="123"/>
-      <c r="H7" s="124"/>
+      <c r="B7" s="127"/>
+      <c r="C7" s="127"/>
+      <c r="D7" s="127"/>
+      <c r="E7" s="127"/>
+      <c r="F7" s="127"/>
+      <c r="G7" s="127"/>
+      <c r="H7" s="128"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="122" t="s">
+      <c r="A8" s="126" t="s">
         <v>115</v>
       </c>
-      <c r="B8" s="123"/>
-      <c r="C8" s="123"/>
-      <c r="D8" s="123"/>
-      <c r="E8" s="123"/>
-      <c r="F8" s="123"/>
-      <c r="G8" s="123"/>
-      <c r="H8" s="124"/>
+      <c r="B8" s="127"/>
+      <c r="C8" s="127"/>
+      <c r="D8" s="127"/>
+      <c r="E8" s="127"/>
+      <c r="F8" s="127"/>
+      <c r="G8" s="127"/>
+      <c r="H8" s="128"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="125" t="s">
+      <c r="A9" s="129" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="125"/>
-      <c r="C9" s="125"/>
-      <c r="D9" s="125"/>
-      <c r="E9" s="125"/>
-      <c r="F9" s="125"/>
-      <c r="G9" s="125"/>
-      <c r="H9" s="125"/>
+      <c r="B9" s="129"/>
+      <c r="C9" s="129"/>
+      <c r="D9" s="129"/>
+      <c r="E9" s="129"/>
+      <c r="F9" s="129"/>
+      <c r="G9" s="129"/>
+      <c r="H9" s="129"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="47">
         <v>1</v>
       </c>
-      <c r="B10" s="121" t="s">
+      <c r="B10" s="125" t="s">
         <v>116</v>
       </c>
-      <c r="C10" s="121"/>
-      <c r="D10" s="121"/>
-      <c r="E10" s="121"/>
-      <c r="F10" s="121"/>
-      <c r="G10" s="121"/>
-      <c r="H10" s="121"/>
+      <c r="C10" s="125"/>
+      <c r="D10" s="125"/>
+      <c r="E10" s="125"/>
+      <c r="F10" s="125"/>
+      <c r="G10" s="125"/>
+      <c r="H10" s="125"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="47">
         <v>2</v>
       </c>
-      <c r="B11" s="121" t="s">
+      <c r="B11" s="125" t="s">
         <v>117</v>
       </c>
-      <c r="C11" s="121"/>
-      <c r="D11" s="121"/>
-      <c r="E11" s="121"/>
-      <c r="F11" s="121"/>
-      <c r="G11" s="121"/>
-      <c r="H11" s="121"/>
+      <c r="C11" s="125"/>
+      <c r="D11" s="125"/>
+      <c r="E11" s="125"/>
+      <c r="F11" s="125"/>
+      <c r="G11" s="125"/>
+      <c r="H11" s="125"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="125" t="s">
+      <c r="A12" s="129" t="s">
         <v>109</v>
       </c>
-      <c r="B12" s="125"/>
-      <c r="C12" s="125"/>
-      <c r="D12" s="125"/>
-      <c r="E12" s="125"/>
-      <c r="F12" s="125"/>
-      <c r="G12" s="125"/>
-      <c r="H12" s="125"/>
+      <c r="B12" s="129"/>
+      <c r="C12" s="129"/>
+      <c r="D12" s="129"/>
+      <c r="E12" s="129"/>
+      <c r="F12" s="129"/>
+      <c r="G12" s="129"/>
+      <c r="H12" s="129"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="47">
         <v>1</v>
       </c>
-      <c r="B13" s="121" t="s">
+      <c r="B13" s="125" t="s">
         <v>118</v>
       </c>
-      <c r="C13" s="121"/>
-      <c r="D13" s="121"/>
-      <c r="E13" s="121"/>
-      <c r="F13" s="121"/>
-      <c r="G13" s="121"/>
-      <c r="H13" s="121"/>
+      <c r="C13" s="125"/>
+      <c r="D13" s="125"/>
+      <c r="E13" s="125"/>
+      <c r="F13" s="125"/>
+      <c r="G13" s="125"/>
+      <c r="H13" s="125"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="47">
         <v>2</v>
       </c>
-      <c r="B14" s="121" t="s">
+      <c r="B14" s="125" t="s">
         <v>119</v>
       </c>
-      <c r="C14" s="121"/>
-      <c r="D14" s="121"/>
-      <c r="E14" s="121"/>
-      <c r="F14" s="121"/>
-      <c r="G14" s="121"/>
-      <c r="H14" s="121"/>
+      <c r="C14" s="125"/>
+      <c r="D14" s="125"/>
+      <c r="E14" s="125"/>
+      <c r="F14" s="125"/>
+      <c r="G14" s="125"/>
+      <c r="H14" s="125"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="47">
         <v>3</v>
       </c>
-      <c r="B15" s="121"/>
-      <c r="C15" s="121"/>
-      <c r="D15" s="121"/>
-      <c r="E15" s="121"/>
-      <c r="F15" s="121"/>
-      <c r="G15" s="121"/>
-      <c r="H15" s="121"/>
+      <c r="B15" s="125"/>
+      <c r="C15" s="125"/>
+      <c r="D15" s="125"/>
+      <c r="E15" s="125"/>
+      <c r="F15" s="125"/>
+      <c r="G15" s="125"/>
+      <c r="H15" s="125"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="47">
         <v>4</v>
       </c>
-      <c r="B16" s="121"/>
-      <c r="C16" s="121"/>
-      <c r="D16" s="121"/>
-      <c r="E16" s="121"/>
-      <c r="F16" s="121"/>
-      <c r="G16" s="121"/>
-      <c r="H16" s="121"/>
+      <c r="B16" s="125"/>
+      <c r="C16" s="125"/>
+      <c r="D16" s="125"/>
+      <c r="E16" s="125"/>
+      <c r="F16" s="125"/>
+      <c r="G16" s="125"/>
+      <c r="H16" s="125"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="47">
         <v>5</v>
       </c>
-      <c r="B17" s="121"/>
-      <c r="C17" s="121"/>
-      <c r="D17" s="121"/>
-      <c r="E17" s="121"/>
-      <c r="F17" s="121"/>
-      <c r="G17" s="121"/>
-      <c r="H17" s="121"/>
+      <c r="B17" s="125"/>
+      <c r="C17" s="125"/>
+      <c r="D17" s="125"/>
+      <c r="E17" s="125"/>
+      <c r="F17" s="125"/>
+      <c r="G17" s="125"/>
+      <c r="H17" s="125"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A18" s="125" t="s">
+      <c r="A18" s="129" t="s">
         <v>120</v>
       </c>
-      <c r="B18" s="125"/>
-      <c r="C18" s="125"/>
-      <c r="D18" s="125"/>
-      <c r="E18" s="125"/>
-      <c r="F18" s="125"/>
-      <c r="G18" s="125"/>
-      <c r="H18" s="125"/>
+      <c r="B18" s="129"/>
+      <c r="C18" s="129"/>
+      <c r="D18" s="129"/>
+      <c r="E18" s="129"/>
+      <c r="F18" s="129"/>
+      <c r="G18" s="129"/>
+      <c r="H18" s="129"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="121" t="s">
+      <c r="A19" s="125" t="s">
         <v>121</v>
       </c>
-      <c r="B19" s="121"/>
-      <c r="C19" s="121"/>
-      <c r="D19" s="121"/>
-      <c r="E19" s="121"/>
-      <c r="F19" s="121"/>
-      <c r="G19" s="121"/>
-      <c r="H19" s="121"/>
+      <c r="B19" s="125"/>
+      <c r="C19" s="125"/>
+      <c r="D19" s="125"/>
+      <c r="E19" s="125"/>
+      <c r="F19" s="125"/>
+      <c r="G19" s="125"/>
+      <c r="H19" s="125"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="121" t="s">
+      <c r="A20" s="125" t="s">
         <v>122</v>
       </c>
-      <c r="B20" s="121"/>
-      <c r="C20" s="121"/>
-      <c r="D20" s="121"/>
-      <c r="E20" s="121"/>
-      <c r="F20" s="121"/>
-      <c r="G20" s="121"/>
-      <c r="H20" s="121"/>
+      <c r="B20" s="125"/>
+      <c r="C20" s="125"/>
+      <c r="D20" s="125"/>
+      <c r="E20" s="125"/>
+      <c r="F20" s="125"/>
+      <c r="G20" s="125"/>
+      <c r="H20" s="125"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="121"/>
-      <c r="B21" s="121"/>
-      <c r="C21" s="121"/>
-      <c r="D21" s="121"/>
-      <c r="E21" s="121"/>
-      <c r="F21" s="121"/>
-      <c r="G21" s="121"/>
-      <c r="H21" s="121"/>
+      <c r="A21" s="125"/>
+      <c r="B21" s="125"/>
+      <c r="C21" s="125"/>
+      <c r="D21" s="125"/>
+      <c r="E21" s="125"/>
+      <c r="F21" s="125"/>
+      <c r="G21" s="125"/>
+      <c r="H21" s="125"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="125" t="s">
+      <c r="A22" s="129" t="s">
         <v>123</v>
       </c>
-      <c r="B22" s="125"/>
-      <c r="C22" s="125"/>
-      <c r="D22" s="125"/>
-      <c r="E22" s="125"/>
-      <c r="F22" s="125"/>
-      <c r="G22" s="125"/>
-      <c r="H22" s="125"/>
+      <c r="B22" s="129"/>
+      <c r="C22" s="129"/>
+      <c r="D22" s="129"/>
+      <c r="E22" s="129"/>
+      <c r="F22" s="129"/>
+      <c r="G22" s="129"/>
+      <c r="H22" s="129"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="121" t="s">
+      <c r="A23" s="125" t="s">
         <v>124</v>
       </c>
-      <c r="B23" s="121"/>
-      <c r="C23" s="121"/>
-      <c r="D23" s="121"/>
-      <c r="E23" s="121"/>
-      <c r="F23" s="121"/>
-      <c r="G23" s="121"/>
-      <c r="H23" s="121"/>
+      <c r="B23" s="125"/>
+      <c r="C23" s="125"/>
+      <c r="D23" s="125"/>
+      <c r="E23" s="125"/>
+      <c r="F23" s="125"/>
+      <c r="G23" s="125"/>
+      <c r="H23" s="125"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A24" s="121"/>
-      <c r="B24" s="121"/>
-      <c r="C24" s="121"/>
-      <c r="D24" s="121"/>
-      <c r="E24" s="121"/>
-      <c r="F24" s="121"/>
-      <c r="G24" s="121"/>
-      <c r="H24" s="121"/>
+      <c r="A24" s="125"/>
+      <c r="B24" s="125"/>
+      <c r="C24" s="125"/>
+      <c r="D24" s="125"/>
+      <c r="E24" s="125"/>
+      <c r="F24" s="125"/>
+      <c r="G24" s="125"/>
+      <c r="H24" s="125"/>
     </row>
     <row r="25" spans="1:8" ht="409.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="47" t="s">
         <v>110</v>
       </c>
-      <c r="B25" s="121"/>
-      <c r="C25" s="121"/>
-      <c r="D25" s="121"/>
-      <c r="E25" s="121"/>
-      <c r="F25" s="121"/>
-      <c r="G25" s="121"/>
-      <c r="H25" s="121"/>
+      <c r="B25" s="125"/>
+      <c r="C25" s="125"/>
+      <c r="D25" s="125"/>
+      <c r="E25" s="125"/>
+      <c r="F25" s="125"/>
+      <c r="G25" s="125"/>
+      <c r="H25" s="125"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="47" t="s">
         <v>111</v>
       </c>
-      <c r="B26" s="121"/>
-      <c r="C26" s="121"/>
-      <c r="D26" s="121"/>
-      <c r="E26" s="121"/>
-      <c r="F26" s="121"/>
-      <c r="G26" s="121"/>
-      <c r="H26" s="121"/>
+      <c r="B26" s="125"/>
+      <c r="C26" s="125"/>
+      <c r="D26" s="125"/>
+      <c r="E26" s="125"/>
+      <c r="F26" s="125"/>
+      <c r="G26" s="125"/>
+      <c r="H26" s="125"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="49"/>
@@ -6601,94 +6601,94 @@
       <c r="C1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="97" t="s">
+      <c r="D1" s="101" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="99"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="103"/>
     </row>
     <row r="2" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="100" t="s">
+      <c r="B2" s="104" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="101"/>
+      <c r="C2" s="105"/>
       <c r="D2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="100" t="s">
+      <c r="E2" s="104" t="s">
         <v>97</v>
       </c>
-      <c r="F2" s="102"/>
-      <c r="G2" s="102"/>
-      <c r="H2" s="103"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="107"/>
     </row>
     <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="104" t="s">
+      <c r="A3" s="108" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="98"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="105"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98"/>
-      <c r="H3" s="99"/>
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="103"/>
     </row>
     <row r="4" spans="1:8" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="19">
         <v>1</v>
       </c>
-      <c r="B4" s="94" t="s">
+      <c r="B4" s="98" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="96"/>
+      <c r="C4" s="99"/>
+      <c r="D4" s="99"/>
+      <c r="E4" s="99"/>
+      <c r="F4" s="99"/>
+      <c r="G4" s="99"/>
+      <c r="H4" s="100"/>
     </row>
     <row r="5" spans="1:8" ht="16.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="20">
         <v>2</v>
       </c>
-      <c r="B5" s="100" t="s">
+      <c r="B5" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="102"/>
-      <c r="D5" s="102"/>
-      <c r="E5" s="102"/>
-      <c r="F5" s="102"/>
-      <c r="G5" s="102"/>
-      <c r="H5" s="103"/>
+      <c r="C5" s="106"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="106"/>
+      <c r="F5" s="106"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="107"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="106" t="s">
+      <c r="A6" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="98"/>
-      <c r="C6" s="98"/>
-      <c r="D6" s="98"/>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98"/>
-      <c r="G6" s="98"/>
-      <c r="H6" s="99"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="102"/>
+      <c r="H6" s="103"/>
     </row>
     <row r="7" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="130" t="s">
+      <c r="A7" s="134" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="95"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="131" t="s">
+      <c r="B7" s="99"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="135" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="112"/>
+      <c r="E7" s="116"/>
       <c r="F7" s="21" t="s">
         <v>20</v>
       </c>
@@ -6703,14 +6703,14 @@
       <c r="A8" s="19">
         <v>1</v>
       </c>
-      <c r="B8" s="94" t="s">
+      <c r="B8" s="98" t="s">
         <v>62</v>
       </c>
-      <c r="C8" s="112"/>
-      <c r="D8" s="94" t="s">
+      <c r="C8" s="116"/>
+      <c r="D8" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E8" s="112"/>
+      <c r="E8" s="116"/>
       <c r="F8" s="46" t="s">
         <v>95</v>
       </c>
@@ -6721,14 +6721,14 @@
       <c r="A9" s="19">
         <v>2</v>
       </c>
-      <c r="B9" s="94" t="s">
+      <c r="B9" s="98" t="s">
         <v>63</v>
       </c>
-      <c r="C9" s="112"/>
-      <c r="D9" s="94" t="s">
+      <c r="C9" s="116"/>
+      <c r="D9" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E9" s="112"/>
+      <c r="E9" s="116"/>
       <c r="F9" s="46" t="s">
         <v>95</v>
       </c>
@@ -6739,14 +6739,14 @@
       <c r="A10" s="19">
         <v>3</v>
       </c>
-      <c r="B10" s="94" t="s">
+      <c r="B10" s="98" t="s">
         <v>68</v>
       </c>
-      <c r="C10" s="112"/>
-      <c r="D10" s="94" t="s">
+      <c r="C10" s="116"/>
+      <c r="D10" s="98" t="s">
         <v>243</v>
       </c>
-      <c r="E10" s="112"/>
+      <c r="E10" s="116"/>
       <c r="F10" s="46" t="s">
         <v>95</v>
       </c>
@@ -6757,14 +6757,14 @@
       <c r="A11" s="19">
         <v>4</v>
       </c>
-      <c r="B11" s="94" t="s">
+      <c r="B11" s="98" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="112"/>
-      <c r="D11" s="94" t="s">
+      <c r="C11" s="116"/>
+      <c r="D11" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E11" s="112"/>
+      <c r="E11" s="116"/>
       <c r="F11" s="46" t="s">
         <v>95</v>
       </c>
@@ -6775,14 +6775,14 @@
       <c r="A12" s="19">
         <v>5</v>
       </c>
-      <c r="B12" s="94" t="s">
+      <c r="B12" s="98" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="112"/>
-      <c r="D12" s="94" t="s">
+      <c r="C12" s="116"/>
+      <c r="D12" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E12" s="112"/>
+      <c r="E12" s="116"/>
       <c r="F12" s="46" t="s">
         <v>95</v>
       </c>
@@ -6793,14 +6793,14 @@
       <c r="A13" s="19">
         <v>6</v>
       </c>
-      <c r="B13" s="94" t="s">
+      <c r="B13" s="98" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="112"/>
-      <c r="D13" s="94" t="s">
+      <c r="C13" s="116"/>
+      <c r="D13" s="98" t="s">
         <v>243</v>
       </c>
-      <c r="E13" s="112"/>
+      <c r="E13" s="116"/>
       <c r="F13" s="46" t="s">
         <v>95</v>
       </c>
@@ -6811,14 +6811,14 @@
       <c r="A14" s="23">
         <v>7</v>
       </c>
-      <c r="B14" s="94" t="s">
+      <c r="B14" s="98" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="111"/>
-      <c r="D14" s="94" t="s">
+      <c r="C14" s="115"/>
+      <c r="D14" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E14" s="112"/>
+      <c r="E14" s="116"/>
       <c r="F14" s="46" t="s">
         <v>95</v>
       </c>
@@ -6829,14 +6829,14 @@
       <c r="A15" s="23">
         <v>8</v>
       </c>
-      <c r="B15" s="94" t="s">
+      <c r="B15" s="98" t="s">
         <v>67</v>
       </c>
-      <c r="C15" s="111"/>
-      <c r="D15" s="94" t="s">
+      <c r="C15" s="115"/>
+      <c r="D15" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E15" s="112"/>
+      <c r="E15" s="116"/>
       <c r="F15" s="46" t="s">
         <v>95</v>
       </c>
@@ -6847,14 +6847,14 @@
       <c r="A16" s="23">
         <v>9</v>
       </c>
-      <c r="B16" s="132" t="s">
+      <c r="B16" s="136" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="133"/>
-      <c r="D16" s="100" t="s">
+      <c r="C16" s="137"/>
+      <c r="D16" s="104" t="s">
         <v>243</v>
       </c>
-      <c r="E16" s="120"/>
+      <c r="E16" s="124"/>
       <c r="F16" s="46" t="s">
         <v>95</v>
       </c>
@@ -6862,22 +6862,22 @@
       <c r="H16" s="25"/>
     </row>
     <row r="17" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="113" t="s">
+      <c r="A17" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="114"/>
-      <c r="C17" s="115" t="s">
+      <c r="B17" s="118"/>
+      <c r="C17" s="119" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="116"/>
+      <c r="D17" s="120"/>
       <c r="E17" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="117">
+      <c r="F17" s="121">
         <v>46227</v>
       </c>
-      <c r="G17" s="118"/>
-      <c r="H17" s="119"/>
+      <c r="G17" s="122"/>
+      <c r="H17" s="123"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -6929,18 +6929,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="88" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
+      <c r="B1" s="88"/>
+      <c r="C1" s="88"/>
       <c r="D1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="85" t="s">
+      <c r="E1" s="89" t="s">
         <v>132</v>
       </c>
-      <c r="F1" s="85"/>
+      <c r="F1" s="89"/>
     </row>
     <row r="2" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="33"/>
@@ -6950,18 +6950,18 @@
       <c r="E2" s="34"/>
     </row>
     <row r="3" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="85" t="s">
+      <c r="A3" s="89" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="85"/>
+      <c r="B3" s="89"/>
       <c r="C3" s="31"/>
       <c r="D3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="85" t="s">
+      <c r="E3" s="89" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="85"/>
+      <c r="F3" s="89"/>
     </row>
     <row r="4" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="7"/>
@@ -6971,44 +6971,44 @@
       <c r="E4" s="7"/>
     </row>
     <row r="5" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="83" t="s">
+      <c r="A5" s="87" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="83"/>
-      <c r="C5" s="78" t="s">
+      <c r="B5" s="87"/>
+      <c r="C5" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="78"/>
-      <c r="E5" s="78"/>
+      <c r="D5" s="82"/>
+      <c r="E5" s="82"/>
     </row>
     <row r="6" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="83" t="s">
+      <c r="A6" s="87" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="83"/>
-      <c r="C6" s="78" t="s">
+      <c r="B6" s="87"/>
+      <c r="C6" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="78"/>
-      <c r="E6" s="78"/>
+      <c r="D6" s="82"/>
+      <c r="E6" s="82"/>
     </row>
     <row r="7" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="83" t="s">
+      <c r="A7" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="83"/>
-      <c r="C7" s="78" t="s">
+      <c r="B7" s="87"/>
+      <c r="C7" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="78"/>
-      <c r="E7" s="78"/>
+      <c r="D7" s="82"/>
+      <c r="E7" s="82"/>
     </row>
     <row r="8" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="79"/>
-      <c r="B8" s="79"/>
-      <c r="C8" s="80"/>
-      <c r="D8" s="80"/>
-      <c r="E8" s="80"/>
+      <c r="A8" s="83"/>
+      <c r="B8" s="83"/>
+      <c r="C8" s="84"/>
+      <c r="D8" s="84"/>
+      <c r="E8" s="84"/>
     </row>
     <row r="9" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="32"/>
@@ -7018,19 +7018,19 @@
       <c r="E9" s="32"/>
     </row>
     <row r="10" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A10" s="81" t="s">
+      <c r="A10" s="85" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="81"/>
-      <c r="C10" s="81"/>
+      <c r="B10" s="85"/>
+      <c r="C10" s="85"/>
       <c r="D10" s="14"/>
       <c r="E10" s="32"/>
     </row>
     <row r="11" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="82" t="s">
+      <c r="A11" s="86" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="82"/>
+      <c r="B11" s="86"/>
       <c r="C11" s="45" t="s">
         <v>95</v>
       </c>
@@ -7038,10 +7038,10 @@
       <c r="E11" s="32"/>
     </row>
     <row r="12" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="82" t="s">
+      <c r="A12" s="86" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="82"/>
+      <c r="B12" s="86"/>
       <c r="C12" s="45" t="s">
         <v>95</v>
       </c>
@@ -7049,10 +7049,10 @@
       <c r="E12" s="32"/>
     </row>
     <row r="13" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A13" s="82" t="s">
+      <c r="A13" s="86" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="82"/>
+      <c r="B13" s="86"/>
       <c r="C13" s="45" t="s">
         <v>95</v>
       </c>
@@ -7060,10 +7060,10 @@
       <c r="E13" s="32"/>
     </row>
     <row r="14" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="91" t="s">
+      <c r="A14" s="95" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="90"/>
+      <c r="B14" s="94"/>
       <c r="C14" s="45" t="s">
         <v>95</v>
       </c>
@@ -7071,10 +7071,10 @@
       <c r="E14" s="32"/>
     </row>
     <row r="15" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A15" s="82" t="s">
+      <c r="A15" s="86" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="82"/>
+      <c r="B15" s="86"/>
       <c r="C15" s="45" t="s">
         <v>95</v>
       </c>
@@ -7082,10 +7082,10 @@
       <c r="E15" s="32"/>
     </row>
     <row r="16" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A16" s="82" t="s">
+      <c r="A16" s="86" t="s">
         <v>53</v>
       </c>
-      <c r="B16" s="82"/>
+      <c r="B16" s="86"/>
       <c r="C16" s="45" t="s">
         <v>95</v>
       </c>
@@ -7140,94 +7140,94 @@
       <c r="C1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="97" t="s">
+      <c r="D1" s="101" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="99"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="103"/>
     </row>
     <row r="2" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="100" t="s">
+      <c r="B2" s="104" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="101"/>
+      <c r="C2" s="105"/>
       <c r="D2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="100" t="s">
+      <c r="E2" s="104" t="s">
         <v>97</v>
       </c>
-      <c r="F2" s="102"/>
-      <c r="G2" s="102"/>
-      <c r="H2" s="103"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="107"/>
     </row>
     <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="104" t="s">
+      <c r="A3" s="108" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="98"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="105"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98"/>
-      <c r="H3" s="99"/>
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="103"/>
     </row>
     <row r="4" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="19">
         <v>1</v>
       </c>
-      <c r="B4" s="94" t="s">
+      <c r="B4" s="98" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="96"/>
+      <c r="C4" s="99"/>
+      <c r="D4" s="99"/>
+      <c r="E4" s="99"/>
+      <c r="F4" s="99"/>
+      <c r="G4" s="99"/>
+      <c r="H4" s="100"/>
     </row>
     <row r="5" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="20">
         <v>2</v>
       </c>
-      <c r="B5" s="100" t="s">
+      <c r="B5" s="104" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="102"/>
-      <c r="D5" s="102"/>
-      <c r="E5" s="102"/>
-      <c r="F5" s="102"/>
-      <c r="G5" s="102"/>
-      <c r="H5" s="103"/>
+      <c r="C5" s="106"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="106"/>
+      <c r="F5" s="106"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="107"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="106" t="s">
+      <c r="A6" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="98"/>
-      <c r="C6" s="98"/>
-      <c r="D6" s="98"/>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98"/>
-      <c r="G6" s="98"/>
-      <c r="H6" s="99"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="102"/>
+      <c r="H6" s="103"/>
     </row>
     <row r="7" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="130" t="s">
+      <c r="A7" s="134" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="95"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="131" t="s">
+      <c r="B7" s="99"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="135" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="112"/>
+      <c r="E7" s="116"/>
       <c r="F7" s="21" t="s">
         <v>20</v>
       </c>
@@ -7242,14 +7242,14 @@
       <c r="A8" s="19">
         <v>1</v>
       </c>
-      <c r="B8" s="94" t="s">
+      <c r="B8" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="111"/>
-      <c r="D8" s="94" t="s">
+      <c r="C8" s="115"/>
+      <c r="D8" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E8" s="112"/>
+      <c r="E8" s="116"/>
       <c r="F8" s="46" t="s">
         <v>95</v>
       </c>
@@ -7260,14 +7260,14 @@
       <c r="A9" s="19">
         <v>2</v>
       </c>
-      <c r="B9" s="94" t="s">
+      <c r="B9" s="98" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="111"/>
-      <c r="D9" s="94" t="s">
+      <c r="C9" s="115"/>
+      <c r="D9" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E9" s="112"/>
+      <c r="E9" s="116"/>
       <c r="F9" s="46" t="s">
         <v>95</v>
       </c>
@@ -7278,14 +7278,14 @@
       <c r="A10" s="19">
         <v>3</v>
       </c>
-      <c r="B10" s="94" t="s">
+      <c r="B10" s="98" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="111"/>
-      <c r="D10" s="94" t="s">
+      <c r="C10" s="115"/>
+      <c r="D10" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E10" s="112"/>
+      <c r="E10" s="116"/>
       <c r="F10" s="46" t="s">
         <v>95</v>
       </c>
@@ -7296,14 +7296,14 @@
       <c r="A11" s="19">
         <v>4</v>
       </c>
-      <c r="B11" s="94" t="s">
+      <c r="B11" s="98" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="111"/>
-      <c r="D11" s="94" t="s">
+      <c r="C11" s="115"/>
+      <c r="D11" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E11" s="112"/>
+      <c r="E11" s="116"/>
       <c r="F11" s="46" t="s">
         <v>95</v>
       </c>
@@ -7314,14 +7314,14 @@
       <c r="A12" s="19">
         <v>5</v>
       </c>
-      <c r="B12" s="94" t="s">
+      <c r="B12" s="98" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="111"/>
-      <c r="D12" s="94" t="s">
+      <c r="C12" s="115"/>
+      <c r="D12" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E12" s="112"/>
+      <c r="E12" s="116"/>
       <c r="F12" s="46" t="s">
         <v>95</v>
       </c>
@@ -7332,14 +7332,14 @@
       <c r="A13" s="19">
         <v>6</v>
       </c>
-      <c r="B13" s="94" t="s">
+      <c r="B13" s="98" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="111"/>
-      <c r="D13" s="94" t="s">
+      <c r="C13" s="115"/>
+      <c r="D13" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E13" s="112"/>
+      <c r="E13" s="116"/>
       <c r="F13" s="46" t="s">
         <v>95</v>
       </c>
@@ -7350,14 +7350,14 @@
       <c r="A14" s="23">
         <v>7</v>
       </c>
-      <c r="B14" s="94" t="s">
+      <c r="B14" s="98" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="111"/>
-      <c r="D14" s="94" t="s">
+      <c r="C14" s="115"/>
+      <c r="D14" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E14" s="112"/>
+      <c r="E14" s="116"/>
       <c r="F14" s="46" t="s">
         <v>95</v>
       </c>
@@ -7368,14 +7368,14 @@
       <c r="A15" s="23">
         <v>8</v>
       </c>
-      <c r="B15" s="94" t="s">
+      <c r="B15" s="98" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="111"/>
-      <c r="D15" s="94" t="s">
+      <c r="C15" s="115"/>
+      <c r="D15" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E15" s="112"/>
+      <c r="E15" s="116"/>
       <c r="F15" s="46" t="s">
         <v>95</v>
       </c>
@@ -7386,14 +7386,14 @@
       <c r="A16" s="23">
         <v>9</v>
       </c>
-      <c r="B16" s="100" t="s">
+      <c r="B16" s="104" t="s">
         <v>210</v>
       </c>
-      <c r="C16" s="120"/>
-      <c r="D16" s="94" t="s">
+      <c r="C16" s="124"/>
+      <c r="D16" s="98" t="s">
         <v>242</v>
       </c>
-      <c r="E16" s="112"/>
+      <c r="E16" s="116"/>
       <c r="F16" s="46" t="s">
         <v>95</v>
       </c>
@@ -7401,22 +7401,22 @@
       <c r="H16" s="25"/>
     </row>
     <row r="17" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="113" t="s">
+      <c r="A17" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="114"/>
-      <c r="C17" s="115" t="s">
+      <c r="B17" s="118"/>
+      <c r="C17" s="119" t="s">
         <v>2</v>
       </c>
-      <c r="D17" s="116"/>
+      <c r="D17" s="120"/>
       <c r="E17" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F17" s="134">
+      <c r="F17" s="138">
         <v>46227</v>
       </c>
-      <c r="G17" s="135"/>
-      <c r="H17" s="136"/>
+      <c r="G17" s="139"/>
+      <c r="H17" s="140"/>
     </row>
     <row r="25" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
@@ -7480,92 +7480,92 @@
       <c r="C1" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="97" t="s">
+      <c r="D1" s="101" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="98"/>
-      <c r="F1" s="98"/>
-      <c r="G1" s="98"/>
-      <c r="H1" s="99"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="103"/>
     </row>
     <row r="2" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="100" t="s">
+      <c r="B2" s="104" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="101"/>
+      <c r="C2" s="105"/>
       <c r="D2" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="100" t="s">
+      <c r="E2" s="104" t="s">
         <v>97</v>
       </c>
-      <c r="F2" s="102"/>
-      <c r="G2" s="102"/>
-      <c r="H2" s="103"/>
+      <c r="F2" s="106"/>
+      <c r="G2" s="106"/>
+      <c r="H2" s="107"/>
     </row>
     <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A3" s="104" t="s">
+      <c r="A3" s="108" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="98"/>
-      <c r="C3" s="98"/>
-      <c r="D3" s="105"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="98"/>
-      <c r="H3" s="99"/>
+      <c r="B3" s="102"/>
+      <c r="C3" s="102"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="102"/>
+      <c r="F3" s="102"/>
+      <c r="G3" s="102"/>
+      <c r="H3" s="103"/>
     </row>
     <row r="4" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="19">
         <v>1</v>
       </c>
-      <c r="B4" s="94" t="s">
+      <c r="B4" s="98" t="s">
         <v>73</v>
       </c>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="95"/>
-      <c r="H4" s="96"/>
+      <c r="C4" s="99"/>
+      <c r="D4" s="99"/>
+      <c r="E4" s="99"/>
+      <c r="F4" s="99"/>
+      <c r="G4" s="99"/>
+      <c r="H4" s="100"/>
     </row>
     <row r="5" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="20">
         <v>2</v>
       </c>
-      <c r="B5" s="100"/>
-      <c r="C5" s="102"/>
-      <c r="D5" s="102"/>
-      <c r="E5" s="102"/>
-      <c r="F5" s="102"/>
-      <c r="G5" s="102"/>
-      <c r="H5" s="103"/>
+      <c r="B5" s="104"/>
+      <c r="C5" s="106"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="106"/>
+      <c r="F5" s="106"/>
+      <c r="G5" s="106"/>
+      <c r="H5" s="107"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A6" s="106" t="s">
+      <c r="A6" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="98"/>
-      <c r="C6" s="98"/>
-      <c r="D6" s="98"/>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98"/>
-      <c r="G6" s="98"/>
-      <c r="H6" s="99"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="102"/>
+      <c r="E6" s="102"/>
+      <c r="F6" s="102"/>
+      <c r="G6" s="102"/>
+      <c r="H6" s="103"/>
     </row>
     <row r="7" spans="1:8" ht="31" x14ac:dyDescent="0.35">
-      <c r="A7" s="130" t="s">
+      <c r="A7" s="134" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="95"/>
-      <c r="C7" s="112"/>
-      <c r="D7" s="131" t="s">
+      <c r="B7" s="99"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="135" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="112"/>
+      <c r="E7" s="116"/>
       <c r="F7" s="21" t="s">
         <v>20</v>
       </c>
@@ -7580,14 +7580,14 @@
       <c r="A8" s="19">
         <v>1</v>
       </c>
-      <c r="B8" s="94" t="s">
+      <c r="B8" s="98" t="s">
         <v>232</v>
       </c>
-      <c r="C8" s="112"/>
-      <c r="D8" s="94" t="s">
+      <c r="C8" s="116"/>
+      <c r="D8" s="98" t="s">
         <v>236</v>
       </c>
-      <c r="E8" s="112"/>
+      <c r="E8" s="116"/>
       <c r="F8" s="46" t="s">
         <v>95</v>
       </c>
@@ -7598,14 +7598,14 @@
       <c r="A9" s="19">
         <v>2</v>
       </c>
-      <c r="B9" s="94" t="s">
+      <c r="B9" s="98" t="s">
         <v>233</v>
       </c>
-      <c r="C9" s="112"/>
-      <c r="D9" s="94" t="s">
+      <c r="C9" s="116"/>
+      <c r="D9" s="98" t="s">
         <v>237</v>
       </c>
-      <c r="E9" s="112"/>
+      <c r="E9" s="116"/>
       <c r="F9" s="46" t="s">
         <v>95</v>
       </c>
@@ -7616,14 +7616,14 @@
       <c r="A10" s="19">
         <v>3</v>
       </c>
-      <c r="B10" s="94" t="s">
+      <c r="B10" s="98" t="s">
         <v>234</v>
       </c>
-      <c r="C10" s="112"/>
-      <c r="D10" s="94" t="s">
+      <c r="C10" s="116"/>
+      <c r="D10" s="98" t="s">
         <v>236</v>
       </c>
-      <c r="E10" s="112"/>
+      <c r="E10" s="116"/>
       <c r="F10" s="46" t="s">
         <v>95</v>
       </c>
@@ -7634,14 +7634,14 @@
       <c r="A11" s="19">
         <v>4</v>
       </c>
-      <c r="B11" s="94" t="s">
+      <c r="B11" s="98" t="s">
         <v>235</v>
       </c>
-      <c r="C11" s="112"/>
-      <c r="D11" s="94" t="s">
+      <c r="C11" s="116"/>
+      <c r="D11" s="98" t="s">
         <v>238</v>
       </c>
-      <c r="E11" s="112"/>
+      <c r="E11" s="116"/>
       <c r="F11" s="46" t="s">
         <v>95</v>
       </c>
@@ -7652,10 +7652,10 @@
       <c r="A12" s="19">
         <v>5</v>
       </c>
-      <c r="B12" s="94"/>
-      <c r="C12" s="112"/>
-      <c r="D12" s="94"/>
-      <c r="E12" s="112"/>
+      <c r="B12" s="98"/>
+      <c r="C12" s="116"/>
+      <c r="D12" s="98"/>
+      <c r="E12" s="116"/>
       <c r="F12" s="21"/>
       <c r="G12" s="21"/>
       <c r="H12" s="22"/>
@@ -7664,10 +7664,10 @@
       <c r="A13" s="19">
         <v>6</v>
       </c>
-      <c r="B13" s="94"/>
-      <c r="C13" s="112"/>
-      <c r="D13" s="94"/>
-      <c r="E13" s="112"/>
+      <c r="B13" s="98"/>
+      <c r="C13" s="116"/>
+      <c r="D13" s="98"/>
+      <c r="E13" s="116"/>
       <c r="F13" s="21"/>
       <c r="G13" s="21"/>
       <c r="H13" s="22"/>
@@ -7676,31 +7676,31 @@
       <c r="A14" s="23">
         <v>7</v>
       </c>
-      <c r="B14" s="132"/>
-      <c r="C14" s="133"/>
-      <c r="D14" s="132"/>
-      <c r="E14" s="133"/>
+      <c r="B14" s="136"/>
+      <c r="C14" s="137"/>
+      <c r="D14" s="136"/>
+      <c r="E14" s="137"/>
       <c r="F14" s="24"/>
       <c r="G14" s="24"/>
       <c r="H14" s="25"/>
     </row>
     <row r="15" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="113" t="s">
+      <c r="A15" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="114"/>
-      <c r="C15" s="115" t="s">
+      <c r="B15" s="118"/>
+      <c r="C15" s="119" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="116"/>
+      <c r="D15" s="120"/>
       <c r="E15" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="F15" s="137">
+      <c r="F15" s="141">
         <v>46228</v>
       </c>
-      <c r="G15" s="138"/>
-      <c r="H15" s="139"/>
+      <c r="G15" s="142"/>
+      <c r="H15" s="143"/>
     </row>
   </sheetData>
   <mergeCells count="27">

</xml_diff>